<commit_message>
Ajuste en ventana de exploracion
</commit_message>
<xml_diff>
--- a/data/Plantilla_LBEn_M1_modelo.xlsx
+++ b/data/Plantilla_LBEn_M1_modelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\gdrive_luisflorez\Mi unidad\PROYECTOS_LF\ProyectosE2\LBEn_EDIF_app\LBEn_APP_Resol016\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DFDC3A-28BC-439E-B4E5-951ED8E40429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{671AE2D4-1184-46E8-A885-52FF099E622D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18690" yWindow="-150" windowWidth="16850" windowHeight="8880" tabRatio="590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16710" yWindow="570" windowWidth="17490" windowHeight="9820" tabRatio="590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="109">
   <si>
     <t>MONITOREO DE DESEMPEÑO ENERGÉTICO</t>
   </si>
@@ -374,6 +374,12 @@
   <si>
     <t xml:space="preserve">Consumo Normalizado y Ajustado
 (kWh) </t>
+  </si>
+  <si>
+    <t>Área útil (m2):</t>
+  </si>
+  <si>
+    <t>Zona Climática:</t>
   </si>
 </sst>
 </file>
@@ -728,7 +734,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -787,7 +793,6 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="17" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1154,25 +1159,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
     </row>
     <row r="2" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
     </row>
     <row r="4" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
     </row>
     <row r="5" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
@@ -1219,47 +1224,47 @@
       </c>
     </row>
     <row r="11" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
     </row>
     <row r="12" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="32" t="s">
+      <c r="C12" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="D12" s="33"/>
+      <c r="D12" s="32"/>
     </row>
     <row r="13" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="33"/>
+      <c r="D13" s="32"/>
     </row>
     <row r="14" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="C14" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="33"/>
+      <c r="D14" s="32"/>
     </row>
     <row r="15" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="33"/>
+      <c r="D15" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1303,54 +1308,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="38" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
       <c r="AC1" s="15"/>
     </row>
     <row r="2" spans="2:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="35"/>
-      <c r="L2" s="35"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
+      <c r="I2" s="34"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
       <c r="AC2" s="16"/>
     </row>
     <row r="3" spans="2:29" x14ac:dyDescent="0.35">
       <c r="AC3" s="16"/>
     </row>
     <row r="4" spans="2:29" ht="44.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
-      <c r="K4" s="31"/>
-      <c r="L4" s="31"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
       <c r="AC4" s="16"/>
     </row>
     <row r="5" spans="2:29" x14ac:dyDescent="0.35">
@@ -1461,123 +1466,132 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
     </row>
     <row r="4" spans="2:13" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="49" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="33"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="32"/>
       <c r="E4" s="13"/>
-      <c r="I4" s="47" t="s">
+      <c r="I4" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="J4" s="48"/>
-      <c r="K4" s="48"/>
-      <c r="L4" s="48"/>
-      <c r="M4" s="48"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47"/>
+      <c r="L4" s="47"/>
+      <c r="M4" s="47"/>
     </row>
     <row r="5" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="49" t="s">
+      <c r="B5" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="28"/>
-      <c r="I5" s="44" t="s">
+      <c r="C5" s="32"/>
+      <c r="D5" s="27"/>
+      <c r="I5" s="43" t="s">
         <v>94</v>
       </c>
-      <c r="J5" s="45"/>
-      <c r="K5" s="29" t="s">
+      <c r="J5" s="44"/>
+      <c r="K5" s="28" t="s">
         <v>95</v>
       </c>
       <c r="L5" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="M5" s="29"/>
+      <c r="M5" s="28"/>
     </row>
     <row r="6" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="43" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="33"/>
-      <c r="D6" s="28"/>
-      <c r="I6" s="44" t="s">
+      <c r="C6" s="32"/>
+      <c r="D6" s="27"/>
+      <c r="I6" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="45"/>
-      <c r="K6" s="29"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="28"/>
       <c r="L6" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="M6" s="29"/>
+      <c r="M6" s="28"/>
     </row>
     <row r="7" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="43" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="33"/>
-      <c r="D7" s="28"/>
-      <c r="I7" s="44" t="s">
+      <c r="C7" s="32"/>
+      <c r="D7" s="27"/>
+      <c r="I7" s="43" t="s">
         <v>53</v>
       </c>
-      <c r="J7" s="45"/>
-      <c r="K7" s="29"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="28"/>
       <c r="L7" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="M7" s="29"/>
+      <c r="M7" s="28"/>
     </row>
     <row r="8" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="D8" s="22"/>
-      <c r="I8" s="44" t="s">
+      <c r="B8" s="43" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="32"/>
+      <c r="D8" s="27"/>
+      <c r="I8" s="43" t="s">
         <v>96</v>
       </c>
-      <c r="J8" s="45"/>
-      <c r="K8" s="29"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="28"/>
       <c r="L8" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="M8" s="29"/>
+      <c r="M8" s="28"/>
     </row>
     <row r="9" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="I9" s="44" t="s">
+      <c r="B9" s="43" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="32"/>
+      <c r="D9" s="27"/>
+      <c r="I9" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="J9" s="45"/>
-      <c r="K9" s="29"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="28"/>
       <c r="L9" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="M9" s="29"/>
+      <c r="M9" s="28"/>
     </row>
     <row r="10" spans="2:13" s="13" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="I10" s="44" t="s">
+      <c r="I10" s="43" t="s">
         <v>55</v>
       </c>
-      <c r="J10" s="45"/>
-      <c r="K10" s="29"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="28"/>
       <c r="L10" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="M10" s="29"/>
+      <c r="M10" s="28"/>
     </row>
     <row r="11" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="2:13" x14ac:dyDescent="0.35">
@@ -1587,20 +1601,20 @@
       <c r="F13" s="13"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B14" s="30" t="s">
+      <c r="B14" s="29" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="31"/>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="31"/>
-      <c r="I14" s="36" t="s">
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="I14" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="31"/>
-      <c r="M14" s="31"/>
+      <c r="J14" s="30"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
+      <c r="M14" s="30"/>
     </row>
     <row r="15" spans="2:13" ht="26" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="6" t="s">
@@ -1638,495 +1652,495 @@
       <c r="B16" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
       <c r="I16" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="J16" s="23"/>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="25"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="24"/>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B17" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
       <c r="I17" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="25"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="24"/>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B18" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
       <c r="I18" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="J18" s="23"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="23"/>
-      <c r="M18" s="25"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="24"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B19" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
       <c r="I19" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="25"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="24"/>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B20" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
       <c r="I20" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
-      <c r="M20" s="25"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="24"/>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B21" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="23"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
       <c r="I21" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="J21" s="23"/>
-      <c r="K21" s="23"/>
-      <c r="L21" s="23"/>
-      <c r="M21" s="25"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="24"/>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B22" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C22" s="23"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
       <c r="I22" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="J22" s="23"/>
-      <c r="K22" s="23"/>
-      <c r="L22" s="23"/>
-      <c r="M22" s="25"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="24"/>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B23" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="23"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
       <c r="I23" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="25"/>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="24"/>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B24" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C24" s="23"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
       <c r="I24" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="J24" s="23"/>
-      <c r="K24" s="23"/>
-      <c r="L24" s="23"/>
-      <c r="M24" s="25"/>
+      <c r="J24" s="22"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="24"/>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B25" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C25" s="23"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
       <c r="I25" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="J25" s="23"/>
-      <c r="K25" s="23"/>
-      <c r="L25" s="23"/>
-      <c r="M25" s="25"/>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="24"/>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B26" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C26" s="23"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
       <c r="I26" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="J26" s="23"/>
-      <c r="K26" s="23"/>
-      <c r="L26" s="23"/>
-      <c r="M26" s="25"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="24"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B27" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C27" s="23"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
       <c r="I27" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="J27" s="23"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="25"/>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+      <c r="M27" s="24"/>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.35">
       <c r="I28" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="J28" s="26"/>
-      <c r="K28" s="26"/>
-      <c r="L28" s="26"/>
-      <c r="M28" s="27"/>
+      <c r="J28" s="25"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="25"/>
+      <c r="M28" s="26"/>
     </row>
     <row r="31" spans="2:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="32" spans="2:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="46" t="s">
+      <c r="B32" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
     </row>
     <row r="33" spans="2:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="42" t="s">
+      <c r="B33" s="41" t="s">
         <v>81</v>
       </c>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="35"/>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
     </row>
     <row r="34" spans="2:5" ht="26" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="41" t="s">
+      <c r="B34" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="C34" s="33"/>
+      <c r="C34" s="32"/>
       <c r="D34" s="12" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B35" s="51"/>
-      <c r="C35" s="51"/>
+      <c r="B35" s="50"/>
+      <c r="C35" s="50"/>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B36" s="51"/>
-      <c r="C36" s="51"/>
+      <c r="B36" s="50"/>
+      <c r="C36" s="50"/>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B37" s="51"/>
-      <c r="C37" s="51"/>
+      <c r="B37" s="50"/>
+      <c r="C37" s="50"/>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B38" s="51"/>
-      <c r="C38" s="51"/>
+      <c r="B38" s="50"/>
+      <c r="C38" s="50"/>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B39" s="51"/>
-      <c r="C39" s="51"/>
+      <c r="B39" s="50"/>
+      <c r="C39" s="50"/>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B40" s="51"/>
-      <c r="C40" s="51"/>
+      <c r="B40" s="50"/>
+      <c r="C40" s="50"/>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B41" s="51"/>
-      <c r="C41" s="51"/>
+      <c r="B41" s="50"/>
+      <c r="C41" s="50"/>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B42" s="51"/>
-      <c r="C42" s="51"/>
+      <c r="B42" s="50"/>
+      <c r="C42" s="50"/>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B43" s="51"/>
-      <c r="C43" s="51"/>
+      <c r="B43" s="50"/>
+      <c r="C43" s="50"/>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B44" s="51"/>
-      <c r="C44" s="51"/>
+      <c r="B44" s="50"/>
+      <c r="C44" s="50"/>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B45" s="51"/>
-      <c r="C45" s="51"/>
+      <c r="B45" s="50"/>
+      <c r="C45" s="50"/>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B46" s="51"/>
-      <c r="C46" s="51"/>
+      <c r="B46" s="50"/>
+      <c r="C46" s="50"/>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B47" s="51"/>
-      <c r="C47" s="51"/>
+      <c r="B47" s="50"/>
+      <c r="C47" s="50"/>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B48" s="51"/>
-      <c r="C48" s="51"/>
+      <c r="B48" s="50"/>
+      <c r="C48" s="50"/>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B49" s="51"/>
-      <c r="C49" s="51"/>
+      <c r="B49" s="50"/>
+      <c r="C49" s="50"/>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B50" s="51"/>
-      <c r="C50" s="51"/>
+      <c r="B50" s="50"/>
+      <c r="C50" s="50"/>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B51" s="51"/>
-      <c r="C51" s="51"/>
+      <c r="B51" s="50"/>
+      <c r="C51" s="50"/>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B52" s="51"/>
-      <c r="C52" s="51"/>
+      <c r="B52" s="50"/>
+      <c r="C52" s="50"/>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B53" s="51"/>
-      <c r="C53" s="51"/>
+      <c r="B53" s="50"/>
+      <c r="C53" s="50"/>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B54" s="51"/>
-      <c r="C54" s="51"/>
+      <c r="B54" s="50"/>
+      <c r="C54" s="50"/>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B55" s="51"/>
-      <c r="C55" s="51"/>
+      <c r="B55" s="50"/>
+      <c r="C55" s="50"/>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B56" s="51"/>
-      <c r="C56" s="51"/>
+      <c r="B56" s="50"/>
+      <c r="C56" s="50"/>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B57" s="51"/>
-      <c r="C57" s="51"/>
+      <c r="B57" s="50"/>
+      <c r="C57" s="50"/>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B58" s="51"/>
-      <c r="C58" s="51"/>
+      <c r="B58" s="50"/>
+      <c r="C58" s="50"/>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B59" s="51"/>
-      <c r="C59" s="51"/>
+      <c r="B59" s="50"/>
+      <c r="C59" s="50"/>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B60" s="51"/>
-      <c r="C60" s="51"/>
+      <c r="B60" s="50"/>
+      <c r="C60" s="50"/>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B61" s="51"/>
-      <c r="C61" s="51"/>
+      <c r="B61" s="50"/>
+      <c r="C61" s="50"/>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B62" s="51"/>
-      <c r="C62" s="51"/>
+      <c r="B62" s="50"/>
+      <c r="C62" s="50"/>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B63" s="51"/>
-      <c r="C63" s="51"/>
+      <c r="B63" s="50"/>
+      <c r="C63" s="50"/>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B64" s="51"/>
-      <c r="C64" s="51"/>
+      <c r="B64" s="50"/>
+      <c r="C64" s="50"/>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B65" s="51"/>
-      <c r="C65" s="51"/>
+      <c r="B65" s="50"/>
+      <c r="C65" s="50"/>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B66" s="51"/>
-      <c r="C66" s="51"/>
+      <c r="B66" s="50"/>
+      <c r="C66" s="50"/>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B67" s="51"/>
-      <c r="C67" s="51"/>
+      <c r="B67" s="50"/>
+      <c r="C67" s="50"/>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B68" s="51"/>
-      <c r="C68" s="51"/>
+      <c r="B68" s="50"/>
+      <c r="C68" s="50"/>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B69" s="51"/>
-      <c r="C69" s="51"/>
+      <c r="B69" s="50"/>
+      <c r="C69" s="50"/>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B70" s="51"/>
-      <c r="C70" s="51"/>
+      <c r="B70" s="50"/>
+      <c r="C70" s="50"/>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B71" s="51"/>
-      <c r="C71" s="51"/>
+      <c r="B71" s="50"/>
+      <c r="C71" s="50"/>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B72" s="51"/>
-      <c r="C72" s="51"/>
+      <c r="B72" s="50"/>
+      <c r="C72" s="50"/>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B73" s="51"/>
-      <c r="C73" s="51"/>
+      <c r="B73" s="50"/>
+      <c r="C73" s="50"/>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B74" s="51"/>
-      <c r="C74" s="51"/>
+      <c r="B74" s="50"/>
+      <c r="C74" s="50"/>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B75" s="51"/>
-      <c r="C75" s="51"/>
+      <c r="B75" s="50"/>
+      <c r="C75" s="50"/>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B76" s="51"/>
-      <c r="C76" s="51"/>
+      <c r="B76" s="50"/>
+      <c r="C76" s="50"/>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B77" s="51"/>
-      <c r="C77" s="51"/>
+      <c r="B77" s="50"/>
+      <c r="C77" s="50"/>
     </row>
     <row r="78" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B78" s="51"/>
-      <c r="C78" s="51"/>
+      <c r="B78" s="50"/>
+      <c r="C78" s="50"/>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B79" s="51"/>
-      <c r="C79" s="51"/>
+      <c r="B79" s="50"/>
+      <c r="C79" s="50"/>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B80" s="51"/>
-      <c r="C80" s="51"/>
+      <c r="B80" s="50"/>
+      <c r="C80" s="50"/>
     </row>
     <row r="81" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B81" s="51"/>
-      <c r="C81" s="51"/>
+      <c r="B81" s="50"/>
+      <c r="C81" s="50"/>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B82" s="51"/>
-      <c r="C82" s="51"/>
+      <c r="B82" s="50"/>
+      <c r="C82" s="50"/>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B83" s="51"/>
-      <c r="C83" s="51"/>
+      <c r="B83" s="50"/>
+      <c r="C83" s="50"/>
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B84" s="51"/>
-      <c r="C84" s="51"/>
+      <c r="B84" s="50"/>
+      <c r="C84" s="50"/>
     </row>
     <row r="85" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B85" s="51"/>
-      <c r="C85" s="51"/>
+      <c r="B85" s="50"/>
+      <c r="C85" s="50"/>
     </row>
     <row r="86" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B86" s="51"/>
-      <c r="C86" s="51"/>
+      <c r="B86" s="50"/>
+      <c r="C86" s="50"/>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B87" s="51"/>
-      <c r="C87" s="51"/>
+      <c r="B87" s="50"/>
+      <c r="C87" s="50"/>
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B88" s="51"/>
-      <c r="C88" s="51"/>
+      <c r="B88" s="50"/>
+      <c r="C88" s="50"/>
     </row>
     <row r="89" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B89" s="51"/>
-      <c r="C89" s="51"/>
+      <c r="B89" s="50"/>
+      <c r="C89" s="50"/>
     </row>
     <row r="90" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B90" s="51"/>
-      <c r="C90" s="51"/>
+      <c r="B90" s="50"/>
+      <c r="C90" s="50"/>
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B91" s="51"/>
-      <c r="C91" s="51"/>
+      <c r="B91" s="50"/>
+      <c r="C91" s="50"/>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B92" s="51"/>
-      <c r="C92" s="51"/>
+      <c r="B92" s="50"/>
+      <c r="C92" s="50"/>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B93" s="51"/>
-      <c r="C93" s="51"/>
+      <c r="B93" s="50"/>
+      <c r="C93" s="50"/>
     </row>
     <row r="94" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B94" s="51"/>
-      <c r="C94" s="51"/>
+      <c r="B94" s="50"/>
+      <c r="C94" s="50"/>
     </row>
     <row r="95" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B95" s="51"/>
-      <c r="C95" s="51"/>
+      <c r="B95" s="50"/>
+      <c r="C95" s="50"/>
     </row>
     <row r="96" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B96" s="51"/>
-      <c r="C96" s="51"/>
+      <c r="B96" s="50"/>
+      <c r="C96" s="50"/>
     </row>
     <row r="97" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B97" s="51"/>
-      <c r="C97" s="51"/>
+      <c r="B97" s="50"/>
+      <c r="C97" s="50"/>
     </row>
     <row r="98" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B98" s="51"/>
-      <c r="C98" s="51"/>
+      <c r="B98" s="50"/>
+      <c r="C98" s="50"/>
     </row>
     <row r="99" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B99" s="51"/>
-      <c r="C99" s="51"/>
+      <c r="B99" s="50"/>
+      <c r="C99" s="50"/>
     </row>
     <row r="100" spans="2:3" x14ac:dyDescent="0.35">
-      <c r="B100" s="51"/>
-      <c r="C100" s="51"/>
+      <c r="B100" s="50"/>
+      <c r="C100" s="50"/>
     </row>
   </sheetData>
-  <mergeCells count="84">
+  <mergeCells count="86">
     <mergeCell ref="B100:C100"/>
     <mergeCell ref="B95:C95"/>
     <mergeCell ref="B96:C96"/>
@@ -2211,6 +2225,8 @@
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B33:E33"/>
     <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2254,82 +2270,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:23" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="52" t="s">
+      <c r="B1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="52"/>
-      <c r="N1" s="52"/>
-      <c r="O1" s="52"/>
-      <c r="P1" s="52"/>
-      <c r="Q1" s="52"/>
-      <c r="R1" s="52"/>
-      <c r="S1" s="52"/>
-      <c r="T1" s="52"/>
-      <c r="U1" s="52"/>
-      <c r="V1" s="52"/>
-      <c r="W1" s="52"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
+      <c r="L1" s="51"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="51"/>
+      <c r="O1" s="51"/>
+      <c r="P1" s="51"/>
+      <c r="Q1" s="51"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="51"/>
+      <c r="V1" s="51"/>
+      <c r="W1" s="51"/>
     </row>
     <row r="2" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="53"/>
-      <c r="N2" s="53"/>
-      <c r="O2" s="53"/>
-      <c r="P2" s="53"/>
-      <c r="Q2" s="53"/>
-      <c r="R2" s="53"/>
-      <c r="S2" s="53"/>
-      <c r="T2" s="53"/>
-      <c r="U2" s="53"/>
-      <c r="V2" s="53"/>
-      <c r="W2" s="53"/>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="52"/>
+      <c r="N2" s="52"/>
+      <c r="O2" s="52"/>
+      <c r="P2" s="52"/>
+      <c r="Q2" s="52"/>
+      <c r="R2" s="52"/>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="52"/>
+      <c r="V2" s="52"/>
+      <c r="W2" s="52"/>
     </row>
     <row r="5" spans="2:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="54" t="s">
+      <c r="B5" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="55"/>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="55"/>
-      <c r="H5" s="55"/>
-      <c r="I5" s="55"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="55"/>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="55"/>
-      <c r="O5" s="55"/>
-      <c r="P5" s="55"/>
-      <c r="Q5" s="55"/>
-      <c r="R5" s="55"/>
-      <c r="S5" s="55"/>
-      <c r="T5" s="55"/>
-      <c r="U5" s="55"/>
-      <c r="V5" s="55"/>
-      <c r="W5" s="55"/>
+      <c r="C5" s="54"/>
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+      <c r="K5" s="54"/>
+      <c r="L5" s="54"/>
+      <c r="M5" s="54"/>
+      <c r="N5" s="54"/>
+      <c r="O5" s="54"/>
+      <c r="P5" s="54"/>
+      <c r="Q5" s="54"/>
+      <c r="R5" s="54"/>
+      <c r="S5" s="54"/>
+      <c r="T5" s="54"/>
+      <c r="U5" s="54"/>
+      <c r="V5" s="54"/>
+      <c r="W5" s="54"/>
     </row>
     <row r="6" spans="2:23" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="17" t="s">

</xml_diff>

<commit_message>
Cambio en posicion de la ventana Monitoreo
</commit_message>
<xml_diff>
--- a/data/Plantilla_LBEn_M1_modelo.xlsx
+++ b/data/Plantilla_LBEn_M1_modelo.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luisa Hernandez\Downloads\LBEn_APP_Resol016\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3775BA-866D-4766-8F45-6A870A233CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB3738E-B633-4B82-8070-64B60E4454BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="590" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="590" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
     <sheet name="Período_Base" sheetId="2" r:id="rId2"/>
-    <sheet name="Modelo_LBEn" sheetId="3" r:id="rId3"/>
-    <sheet name="Monitoreo" sheetId="4" r:id="rId4"/>
+    <sheet name="Monitoreo" sheetId="4" r:id="rId3"/>
+    <sheet name="Modelo_LBEn" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
 </workbook>
@@ -376,7 +376,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -828,14 +828,8 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -856,8 +850,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1136,7 +1136,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -1145,28 +1145,28 @@
     <col min="5" max="5" width="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="31.5" customHeight="1">
+    <row r="1" spans="2:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="33" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="34"/>
       <c r="D1" s="34"/>
     </row>
-    <row r="2" spans="2:4" ht="18" customHeight="1">
+    <row r="2" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="36" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="34"/>
       <c r="D2" s="34"/>
     </row>
-    <row r="4" spans="2:4" ht="19.5" customHeight="1">
+    <row r="4" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="35" t="s">
         <v>20</v>
       </c>
       <c r="C4" s="30"/>
       <c r="D4" s="30"/>
     </row>
-    <row r="5" spans="2:4" ht="25" customHeight="1">
+    <row r="5" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
@@ -1177,7 +1177,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="36" customHeight="1">
+    <row r="6" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="6" t="s">
         <v>24</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="37.5" customHeight="1">
+    <row r="7" spans="2:4" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>27</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="25" customHeight="1">
+    <row r="8" spans="2:4" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
         <v>30</v>
       </c>
@@ -1210,14 +1210,14 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="19.5" customHeight="1">
+    <row r="11" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="29" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="30"/>
       <c r="D11" s="30"/>
     </row>
-    <row r="12" spans="2:4" ht="18" customHeight="1">
+    <row r="12" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>34</v>
       </c>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D12" s="32"/>
     </row>
-    <row r="13" spans="2:4" ht="18" customHeight="1">
+    <row r="13" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="1" t="s">
         <v>36</v>
       </c>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="D13" s="32"/>
     </row>
-    <row r="14" spans="2:4" ht="18" customHeight="1">
+    <row r="14" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="1" t="s">
         <v>38</v>
       </c>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="D14" s="32"/>
     </row>
-    <row r="15" spans="2:4" ht="18" customHeight="1">
+    <row r="15" spans="2:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="1" t="s">
         <v>40</v>
       </c>
@@ -1272,7 +1272,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:AC7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="9.7265625" bestFit="1" customWidth="1"/>
@@ -1294,7 +1294,7 @@
     <col min="22" max="22" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:29" ht="27.75" customHeight="1">
+    <row r="1" spans="2:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="38" t="s">
         <v>42</v>
       </c>
@@ -1310,7 +1310,7 @@
       <c r="L1" s="34"/>
       <c r="AC1" s="15"/>
     </row>
-    <row r="2" spans="2:29" ht="15.75" customHeight="1">
+    <row r="2" spans="2:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="37" t="s">
         <v>43</v>
       </c>
@@ -1326,10 +1326,10 @@
       <c r="L2" s="34"/>
       <c r="AC2" s="16"/>
     </row>
-    <row r="3" spans="2:29">
+    <row r="3" spans="2:29" x14ac:dyDescent="0.35">
       <c r="AC3" s="16"/>
     </row>
-    <row r="4" spans="2:29" ht="44.5" customHeight="1">
+    <row r="4" spans="2:29" ht="44.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="39" t="s">
         <v>44</v>
       </c>
@@ -1345,10 +1345,10 @@
       <c r="L4" s="30"/>
       <c r="AC4" s="16"/>
     </row>
-    <row r="5" spans="2:29">
+    <row r="5" spans="2:29" x14ac:dyDescent="0.35">
       <c r="S5" s="16"/>
     </row>
-    <row r="6" spans="2:29" ht="36" customHeight="1">
+    <row r="6" spans="2:29" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="17" t="s">
         <v>3</v>
       </c>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="S6" s="16"/>
     </row>
-    <row r="7" spans="2:29" ht="15.75" customHeight="1">
+    <row r="7" spans="2:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="14" t="s">
         <v>14</v>
       </c>
@@ -1433,797 +1433,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B1:M100"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="11.6328125" customWidth="1"/>
-    <col min="3" max="3" width="12.453125" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="26" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="3" customWidth="1"/>
-    <col min="9" max="9" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="22" customWidth="1"/>
-    <col min="12" max="12" width="26" customWidth="1"/>
-    <col min="13" max="13" width="26.6328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:13" ht="27.75" customHeight="1">
-      <c r="B1" s="38" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-    </row>
-    <row r="2" spans="2:13" ht="18" customHeight="1">
-      <c r="B2" s="42" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-    </row>
-    <row r="4" spans="2:13" ht="35" customHeight="1">
-      <c r="B4" s="49" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="13"/>
-      <c r="I4" s="46" t="s">
-        <v>48</v>
-      </c>
-      <c r="J4" s="47"/>
-      <c r="K4" s="47"/>
-      <c r="L4" s="47"/>
-      <c r="M4" s="47"/>
-    </row>
-    <row r="5" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1">
-      <c r="B5" s="48" t="s">
-        <v>49</v>
-      </c>
-      <c r="C5" s="32"/>
-      <c r="D5" s="27"/>
-      <c r="I5" s="43" t="s">
-        <v>94</v>
-      </c>
-      <c r="J5" s="44"/>
-      <c r="K5" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="L5" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="M5" s="28"/>
-    </row>
-    <row r="6" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1">
-      <c r="B6" s="43" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="32"/>
-      <c r="D6" s="27"/>
-      <c r="I6" s="43" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="44"/>
-      <c r="K6" s="28"/>
-      <c r="L6" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="M6" s="28"/>
-    </row>
-    <row r="7" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1">
-      <c r="B7" s="43" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" s="32"/>
-      <c r="D7" s="27"/>
-      <c r="I7" s="43" t="s">
-        <v>53</v>
-      </c>
-      <c r="J7" s="44"/>
-      <c r="K7" s="28"/>
-      <c r="L7" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="M7" s="28"/>
-    </row>
-    <row r="8" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1">
-      <c r="B8" s="43" t="s">
-        <v>106</v>
-      </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="27"/>
-      <c r="I8" s="43" t="s">
-        <v>95</v>
-      </c>
-      <c r="J8" s="44"/>
-      <c r="K8" s="28"/>
-      <c r="L8" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="M8" s="28"/>
-    </row>
-    <row r="9" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1">
-      <c r="B9" s="43" t="s">
-        <v>105</v>
-      </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="27"/>
-      <c r="I9" s="43" t="s">
-        <v>57</v>
-      </c>
-      <c r="J9" s="44"/>
-      <c r="K9" s="28"/>
-      <c r="L9" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="M9" s="28"/>
-    </row>
-    <row r="10" spans="2:13" s="13" customFormat="1" ht="34" customHeight="1">
-      <c r="I10" s="43" t="s">
-        <v>55</v>
-      </c>
-      <c r="J10" s="44"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="M10" s="28"/>
-    </row>
-    <row r="11" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1"/>
-    <row r="12" spans="2:13">
-      <c r="F12" s="13"/>
-    </row>
-    <row r="13" spans="2:13">
-      <c r="F13" s="13"/>
-    </row>
-    <row r="14" spans="2:13">
-      <c r="B14" s="29" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="I14" s="35" t="s">
-        <v>60</v>
-      </c>
-      <c r="J14" s="30"/>
-      <c r="K14" s="30"/>
-      <c r="L14" s="30"/>
-      <c r="M14" s="30"/>
-    </row>
-    <row r="15" spans="2:13" ht="26" customHeight="1">
-      <c r="B15" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="I15" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="J15" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="K15" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="L15" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="2:13">
-      <c r="B16" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C16" s="22"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="I16" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="24"/>
-    </row>
-    <row r="17" spans="2:13">
-      <c r="B17" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="I17" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="24"/>
-    </row>
-    <row r="18" spans="2:13">
-      <c r="B18" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C18" s="22"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="I18" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="24"/>
-    </row>
-    <row r="19" spans="2:13">
-      <c r="B19" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C19" s="22"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="I19" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="24"/>
-    </row>
-    <row r="20" spans="2:13">
-      <c r="B20" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="I20" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="24"/>
-    </row>
-    <row r="21" spans="2:13">
-      <c r="B21" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
-      <c r="I21" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="24"/>
-    </row>
-    <row r="22" spans="2:13">
-      <c r="B22" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
-      <c r="I22" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="24"/>
-    </row>
-    <row r="23" spans="2:13">
-      <c r="B23" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="23"/>
-      <c r="I23" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="24"/>
-    </row>
-    <row r="24" spans="2:13">
-      <c r="B24" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C24" s="22"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
-      <c r="I24" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="24"/>
-    </row>
-    <row r="25" spans="2:13">
-      <c r="B25" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C25" s="22"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="23"/>
-      <c r="I25" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="24"/>
-    </row>
-    <row r="26" spans="2:13">
-      <c r="B26" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
-      <c r="I26" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="J26" s="22"/>
-      <c r="K26" s="22"/>
-      <c r="L26" s="22"/>
-      <c r="M26" s="24"/>
-    </row>
-    <row r="27" spans="2:13">
-      <c r="B27" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="I27" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="24"/>
-    </row>
-    <row r="28" spans="2:13">
-      <c r="I28" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="J28" s="25"/>
-      <c r="K28" s="25"/>
-      <c r="L28" s="25"/>
-      <c r="M28" s="26"/>
-    </row>
-    <row r="31" spans="2:13" ht="19.5" customHeight="1"/>
-    <row r="32" spans="2:13" ht="19.5" customHeight="1">
-      <c r="B32" s="45" t="s">
-        <v>80</v>
-      </c>
-      <c r="C32" s="34"/>
-      <c r="D32" s="34"/>
-      <c r="E32" s="34"/>
-    </row>
-    <row r="33" spans="2:5" ht="27.75" customHeight="1">
-      <c r="B33" s="41" t="s">
-        <v>81</v>
-      </c>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-    </row>
-    <row r="34" spans="2:5" ht="26" customHeight="1">
-      <c r="B34" s="40" t="s">
-        <v>3</v>
-      </c>
-      <c r="C34" s="32"/>
-      <c r="D34" s="12" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5">
-      <c r="B35" s="50"/>
-      <c r="C35" s="50"/>
-    </row>
-    <row r="36" spans="2:5">
-      <c r="B36" s="50"/>
-      <c r="C36" s="50"/>
-    </row>
-    <row r="37" spans="2:5">
-      <c r="B37" s="50"/>
-      <c r="C37" s="50"/>
-    </row>
-    <row r="38" spans="2:5">
-      <c r="B38" s="50"/>
-      <c r="C38" s="50"/>
-    </row>
-    <row r="39" spans="2:5">
-      <c r="B39" s="50"/>
-      <c r="C39" s="50"/>
-    </row>
-    <row r="40" spans="2:5">
-      <c r="B40" s="50"/>
-      <c r="C40" s="50"/>
-    </row>
-    <row r="41" spans="2:5">
-      <c r="B41" s="50"/>
-      <c r="C41" s="50"/>
-    </row>
-    <row r="42" spans="2:5">
-      <c r="B42" s="50"/>
-      <c r="C42" s="50"/>
-    </row>
-    <row r="43" spans="2:5">
-      <c r="B43" s="50"/>
-      <c r="C43" s="50"/>
-    </row>
-    <row r="44" spans="2:5">
-      <c r="B44" s="50"/>
-      <c r="C44" s="50"/>
-    </row>
-    <row r="45" spans="2:5">
-      <c r="B45" s="50"/>
-      <c r="C45" s="50"/>
-    </row>
-    <row r="46" spans="2:5">
-      <c r="B46" s="50"/>
-      <c r="C46" s="50"/>
-    </row>
-    <row r="47" spans="2:5">
-      <c r="B47" s="50"/>
-      <c r="C47" s="50"/>
-    </row>
-    <row r="48" spans="2:5">
-      <c r="B48" s="50"/>
-      <c r="C48" s="50"/>
-    </row>
-    <row r="49" spans="2:3">
-      <c r="B49" s="50"/>
-      <c r="C49" s="50"/>
-    </row>
-    <row r="50" spans="2:3">
-      <c r="B50" s="50"/>
-      <c r="C50" s="50"/>
-    </row>
-    <row r="51" spans="2:3">
-      <c r="B51" s="50"/>
-      <c r="C51" s="50"/>
-    </row>
-    <row r="52" spans="2:3">
-      <c r="B52" s="50"/>
-      <c r="C52" s="50"/>
-    </row>
-    <row r="53" spans="2:3">
-      <c r="B53" s="50"/>
-      <c r="C53" s="50"/>
-    </row>
-    <row r="54" spans="2:3">
-      <c r="B54" s="50"/>
-      <c r="C54" s="50"/>
-    </row>
-    <row r="55" spans="2:3">
-      <c r="B55" s="50"/>
-      <c r="C55" s="50"/>
-    </row>
-    <row r="56" spans="2:3">
-      <c r="B56" s="50"/>
-      <c r="C56" s="50"/>
-    </row>
-    <row r="57" spans="2:3">
-      <c r="B57" s="50"/>
-      <c r="C57" s="50"/>
-    </row>
-    <row r="58" spans="2:3">
-      <c r="B58" s="50"/>
-      <c r="C58" s="50"/>
-    </row>
-    <row r="59" spans="2:3">
-      <c r="B59" s="50"/>
-      <c r="C59" s="50"/>
-    </row>
-    <row r="60" spans="2:3">
-      <c r="B60" s="50"/>
-      <c r="C60" s="50"/>
-    </row>
-    <row r="61" spans="2:3">
-      <c r="B61" s="50"/>
-      <c r="C61" s="50"/>
-    </row>
-    <row r="62" spans="2:3">
-      <c r="B62" s="50"/>
-      <c r="C62" s="50"/>
-    </row>
-    <row r="63" spans="2:3">
-      <c r="B63" s="50"/>
-      <c r="C63" s="50"/>
-    </row>
-    <row r="64" spans="2:3">
-      <c r="B64" s="50"/>
-      <c r="C64" s="50"/>
-    </row>
-    <row r="65" spans="2:3">
-      <c r="B65" s="50"/>
-      <c r="C65" s="50"/>
-    </row>
-    <row r="66" spans="2:3">
-      <c r="B66" s="50"/>
-      <c r="C66" s="50"/>
-    </row>
-    <row r="67" spans="2:3">
-      <c r="B67" s="50"/>
-      <c r="C67" s="50"/>
-    </row>
-    <row r="68" spans="2:3">
-      <c r="B68" s="50"/>
-      <c r="C68" s="50"/>
-    </row>
-    <row r="69" spans="2:3">
-      <c r="B69" s="50"/>
-      <c r="C69" s="50"/>
-    </row>
-    <row r="70" spans="2:3">
-      <c r="B70" s="50"/>
-      <c r="C70" s="50"/>
-    </row>
-    <row r="71" spans="2:3">
-      <c r="B71" s="50"/>
-      <c r="C71" s="50"/>
-    </row>
-    <row r="72" spans="2:3">
-      <c r="B72" s="50"/>
-      <c r="C72" s="50"/>
-    </row>
-    <row r="73" spans="2:3">
-      <c r="B73" s="50"/>
-      <c r="C73" s="50"/>
-    </row>
-    <row r="74" spans="2:3">
-      <c r="B74" s="50"/>
-      <c r="C74" s="50"/>
-    </row>
-    <row r="75" spans="2:3">
-      <c r="B75" s="50"/>
-      <c r="C75" s="50"/>
-    </row>
-    <row r="76" spans="2:3">
-      <c r="B76" s="50"/>
-      <c r="C76" s="50"/>
-    </row>
-    <row r="77" spans="2:3">
-      <c r="B77" s="50"/>
-      <c r="C77" s="50"/>
-    </row>
-    <row r="78" spans="2:3">
-      <c r="B78" s="50"/>
-      <c r="C78" s="50"/>
-    </row>
-    <row r="79" spans="2:3">
-      <c r="B79" s="50"/>
-      <c r="C79" s="50"/>
-    </row>
-    <row r="80" spans="2:3">
-      <c r="B80" s="50"/>
-      <c r="C80" s="50"/>
-    </row>
-    <row r="81" spans="2:3">
-      <c r="B81" s="50"/>
-      <c r="C81" s="50"/>
-    </row>
-    <row r="82" spans="2:3">
-      <c r="B82" s="50"/>
-      <c r="C82" s="50"/>
-    </row>
-    <row r="83" spans="2:3">
-      <c r="B83" s="50"/>
-      <c r="C83" s="50"/>
-    </row>
-    <row r="84" spans="2:3">
-      <c r="B84" s="50"/>
-      <c r="C84" s="50"/>
-    </row>
-    <row r="85" spans="2:3">
-      <c r="B85" s="50"/>
-      <c r="C85" s="50"/>
-    </row>
-    <row r="86" spans="2:3">
-      <c r="B86" s="50"/>
-      <c r="C86" s="50"/>
-    </row>
-    <row r="87" spans="2:3">
-      <c r="B87" s="50"/>
-      <c r="C87" s="50"/>
-    </row>
-    <row r="88" spans="2:3">
-      <c r="B88" s="50"/>
-      <c r="C88" s="50"/>
-    </row>
-    <row r="89" spans="2:3">
-      <c r="B89" s="50"/>
-      <c r="C89" s="50"/>
-    </row>
-    <row r="90" spans="2:3">
-      <c r="B90" s="50"/>
-      <c r="C90" s="50"/>
-    </row>
-    <row r="91" spans="2:3">
-      <c r="B91" s="50"/>
-      <c r="C91" s="50"/>
-    </row>
-    <row r="92" spans="2:3">
-      <c r="B92" s="50"/>
-      <c r="C92" s="50"/>
-    </row>
-    <row r="93" spans="2:3">
-      <c r="B93" s="50"/>
-      <c r="C93" s="50"/>
-    </row>
-    <row r="94" spans="2:3">
-      <c r="B94" s="50"/>
-      <c r="C94" s="50"/>
-    </row>
-    <row r="95" spans="2:3">
-      <c r="B95" s="50"/>
-      <c r="C95" s="50"/>
-    </row>
-    <row r="96" spans="2:3">
-      <c r="B96" s="50"/>
-      <c r="C96" s="50"/>
-    </row>
-    <row r="97" spans="2:3">
-      <c r="B97" s="50"/>
-      <c r="C97" s="50"/>
-    </row>
-    <row r="98" spans="2:3">
-      <c r="B98" s="50"/>
-      <c r="C98" s="50"/>
-    </row>
-    <row r="99" spans="2:3">
-      <c r="B99" s="50"/>
-      <c r="C99" s="50"/>
-    </row>
-    <row r="100" spans="2:3">
-      <c r="B100" s="50"/>
-      <c r="C100" s="50"/>
-    </row>
-  </sheetData>
-  <mergeCells count="86">
-    <mergeCell ref="B100:C100"/>
-    <mergeCell ref="B95:C95"/>
-    <mergeCell ref="B96:C96"/>
-    <mergeCell ref="B97:C97"/>
-    <mergeCell ref="B98:C98"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="B90:C90"/>
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="B92:C92"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B94:C94"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B87:C87"/>
-    <mergeCell ref="B88:C88"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B67:C67"/>
-    <mergeCell ref="B68:C68"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="I14:M14"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I9:J9"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="I4:M4"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B1:W7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -2256,7 +1468,7 @@
     <col min="33" max="33" width="21.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:23" ht="27.75" customHeight="1">
+    <row r="1" spans="2:23" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="51" t="s">
         <v>0</v>
       </c>
@@ -2282,7 +1494,7 @@
       <c r="V1" s="51"/>
       <c r="W1" s="51"/>
     </row>
-    <row r="2" spans="2:23" ht="15.75" customHeight="1">
+    <row r="2" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="52" t="s">
         <v>1</v>
       </c>
@@ -2308,7 +1520,7 @@
       <c r="V2" s="52"/>
       <c r="W2" s="52"/>
     </row>
-    <row r="5" spans="2:23" ht="19.5" customHeight="1">
+    <row r="5" spans="2:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="53" t="s">
         <v>2</v>
       </c>
@@ -2334,7 +1546,7 @@
       <c r="V5" s="54"/>
       <c r="W5" s="54"/>
     </row>
-    <row r="6" spans="2:23" ht="56.5" customHeight="1">
+    <row r="6" spans="2:23" ht="56.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="17" t="s">
         <v>3</v>
       </c>
@@ -2402,7 +1614,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="7" spans="2:23" ht="15.75" customHeight="1">
+    <row r="7" spans="2:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="14" t="s">
         <v>14</v>
       </c>
@@ -2479,4 +1691,792 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="B1:M100"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="2" width="11.6328125" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="3" customWidth="1"/>
+    <col min="9" max="9" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="26" customWidth="1"/>
+    <col min="13" max="13" width="26.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+    </row>
+    <row r="2" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="50" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+    </row>
+    <row r="4" spans="2:13" ht="35" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="47" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="13"/>
+      <c r="I4" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" s="45"/>
+      <c r="K4" s="45"/>
+      <c r="L4" s="45"/>
+      <c r="M4" s="45"/>
+    </row>
+    <row r="5" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="46" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="32"/>
+      <c r="D5" s="27"/>
+      <c r="I5" s="41" t="s">
+        <v>94</v>
+      </c>
+      <c r="J5" s="42"/>
+      <c r="K5" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="L5" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="M5" s="28"/>
+    </row>
+    <row r="6" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="41" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="32"/>
+      <c r="D6" s="27"/>
+      <c r="I6" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="42"/>
+      <c r="K6" s="28"/>
+      <c r="L6" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="M6" s="28"/>
+    </row>
+    <row r="7" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="32"/>
+      <c r="D7" s="27"/>
+      <c r="I7" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" s="42"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M7" s="28"/>
+    </row>
+    <row r="8" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="32"/>
+      <c r="D8" s="27"/>
+      <c r="I8" s="41" t="s">
+        <v>95</v>
+      </c>
+      <c r="J8" s="42"/>
+      <c r="K8" s="28"/>
+      <c r="L8" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="M8" s="28"/>
+    </row>
+    <row r="9" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="32"/>
+      <c r="D9" s="27"/>
+      <c r="I9" s="41" t="s">
+        <v>57</v>
+      </c>
+      <c r="J9" s="42"/>
+      <c r="K9" s="28"/>
+      <c r="L9" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="M9" s="28"/>
+    </row>
+    <row r="10" spans="2:13" s="13" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="I10" s="41" t="s">
+        <v>55</v>
+      </c>
+      <c r="J10" s="42"/>
+      <c r="K10" s="28"/>
+      <c r="L10" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="M10" s="28"/>
+    </row>
+    <row r="11" spans="2:13" s="13" customFormat="1" ht="24.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="F12" s="13"/>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="F13" s="13"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B14" s="29" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="I14" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="J14" s="30"/>
+      <c r="K14" s="30"/>
+      <c r="L14" s="30"/>
+      <c r="M14" s="30"/>
+    </row>
+    <row r="15" spans="2:13" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="J15" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="L15" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B16" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="22"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="I16" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="24"/>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B17" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C17" s="22"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="I17" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="24"/>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B18" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="22"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="I18" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="24"/>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B19" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="22"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="23"/>
+      <c r="I19" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="24"/>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B20" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="22"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="23"/>
+      <c r="I20" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="24"/>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B21" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="22"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="23"/>
+      <c r="I21" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="24"/>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B22" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C22" s="22"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="I22" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="24"/>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B23" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="22"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="23"/>
+      <c r="I23" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="24"/>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B24" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="22"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="23"/>
+      <c r="I24" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="J24" s="22"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="24"/>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B25" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="22"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="I25" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="24"/>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B26" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="22"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="I26" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="24"/>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B27" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="22"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="I27" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+      <c r="M27" s="24"/>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="I28" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="J28" s="25"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="25"/>
+      <c r="M28" s="26"/>
+    </row>
+    <row r="31" spans="2:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="2:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="43" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+    </row>
+    <row r="33" spans="2:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" s="34"/>
+      <c r="D33" s="34"/>
+      <c r="E33" s="34"/>
+    </row>
+    <row r="34" spans="2:5" ht="26" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="48" t="s">
+        <v>3</v>
+      </c>
+      <c r="C34" s="32"/>
+      <c r="D34" s="12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B35" s="40"/>
+      <c r="C35" s="40"/>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B36" s="40"/>
+      <c r="C36" s="40"/>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B37" s="40"/>
+      <c r="C37" s="40"/>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B38" s="40"/>
+      <c r="C38" s="40"/>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B39" s="40"/>
+      <c r="C39" s="40"/>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B40" s="40"/>
+      <c r="C40" s="40"/>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B41" s="40"/>
+      <c r="C41" s="40"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B42" s="40"/>
+      <c r="C42" s="40"/>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B43" s="40"/>
+      <c r="C43" s="40"/>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B44" s="40"/>
+      <c r="C44" s="40"/>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B45" s="40"/>
+      <c r="C45" s="40"/>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B46" s="40"/>
+      <c r="C46" s="40"/>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B47" s="40"/>
+      <c r="C47" s="40"/>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B48" s="40"/>
+      <c r="C48" s="40"/>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B49" s="40"/>
+      <c r="C49" s="40"/>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B50" s="40"/>
+      <c r="C50" s="40"/>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B51" s="40"/>
+      <c r="C51" s="40"/>
+    </row>
+    <row r="52" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B52" s="40"/>
+      <c r="C52" s="40"/>
+    </row>
+    <row r="53" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B53" s="40"/>
+      <c r="C53" s="40"/>
+    </row>
+    <row r="54" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B54" s="40"/>
+      <c r="C54" s="40"/>
+    </row>
+    <row r="55" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B55" s="40"/>
+      <c r="C55" s="40"/>
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B56" s="40"/>
+      <c r="C56" s="40"/>
+    </row>
+    <row r="57" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B57" s="40"/>
+      <c r="C57" s="40"/>
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B58" s="40"/>
+      <c r="C58" s="40"/>
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B59" s="40"/>
+      <c r="C59" s="40"/>
+    </row>
+    <row r="60" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B60" s="40"/>
+      <c r="C60" s="40"/>
+    </row>
+    <row r="61" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B61" s="40"/>
+      <c r="C61" s="40"/>
+    </row>
+    <row r="62" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B62" s="40"/>
+      <c r="C62" s="40"/>
+    </row>
+    <row r="63" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B63" s="40"/>
+      <c r="C63" s="40"/>
+    </row>
+    <row r="64" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B64" s="40"/>
+      <c r="C64" s="40"/>
+    </row>
+    <row r="65" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B65" s="40"/>
+      <c r="C65" s="40"/>
+    </row>
+    <row r="66" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B66" s="40"/>
+      <c r="C66" s="40"/>
+    </row>
+    <row r="67" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B67" s="40"/>
+      <c r="C67" s="40"/>
+    </row>
+    <row r="68" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B68" s="40"/>
+      <c r="C68" s="40"/>
+    </row>
+    <row r="69" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B69" s="40"/>
+      <c r="C69" s="40"/>
+    </row>
+    <row r="70" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B70" s="40"/>
+      <c r="C70" s="40"/>
+    </row>
+    <row r="71" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B71" s="40"/>
+      <c r="C71" s="40"/>
+    </row>
+    <row r="72" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B72" s="40"/>
+      <c r="C72" s="40"/>
+    </row>
+    <row r="73" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B73" s="40"/>
+      <c r="C73" s="40"/>
+    </row>
+    <row r="74" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B74" s="40"/>
+      <c r="C74" s="40"/>
+    </row>
+    <row r="75" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B75" s="40"/>
+      <c r="C75" s="40"/>
+    </row>
+    <row r="76" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B76" s="40"/>
+      <c r="C76" s="40"/>
+    </row>
+    <row r="77" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B77" s="40"/>
+      <c r="C77" s="40"/>
+    </row>
+    <row r="78" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B78" s="40"/>
+      <c r="C78" s="40"/>
+    </row>
+    <row r="79" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B79" s="40"/>
+      <c r="C79" s="40"/>
+    </row>
+    <row r="80" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B80" s="40"/>
+      <c r="C80" s="40"/>
+    </row>
+    <row r="81" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B81" s="40"/>
+      <c r="C81" s="40"/>
+    </row>
+    <row r="82" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B82" s="40"/>
+      <c r="C82" s="40"/>
+    </row>
+    <row r="83" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B83" s="40"/>
+      <c r="C83" s="40"/>
+    </row>
+    <row r="84" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B84" s="40"/>
+      <c r="C84" s="40"/>
+    </row>
+    <row r="85" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B85" s="40"/>
+      <c r="C85" s="40"/>
+    </row>
+    <row r="86" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B86" s="40"/>
+      <c r="C86" s="40"/>
+    </row>
+    <row r="87" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B87" s="40"/>
+      <c r="C87" s="40"/>
+    </row>
+    <row r="88" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B88" s="40"/>
+      <c r="C88" s="40"/>
+    </row>
+    <row r="89" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B89" s="40"/>
+      <c r="C89" s="40"/>
+    </row>
+    <row r="90" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B90" s="40"/>
+      <c r="C90" s="40"/>
+    </row>
+    <row r="91" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B91" s="40"/>
+      <c r="C91" s="40"/>
+    </row>
+    <row r="92" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B92" s="40"/>
+      <c r="C92" s="40"/>
+    </row>
+    <row r="93" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B93" s="40"/>
+      <c r="C93" s="40"/>
+    </row>
+    <row r="94" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B94" s="40"/>
+      <c r="C94" s="40"/>
+    </row>
+    <row r="95" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B95" s="40"/>
+      <c r="C95" s="40"/>
+    </row>
+    <row r="96" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B96" s="40"/>
+      <c r="C96" s="40"/>
+    </row>
+    <row r="97" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B97" s="40"/>
+      <c r="C97" s="40"/>
+    </row>
+    <row r="98" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B98" s="40"/>
+      <c r="C98" s="40"/>
+    </row>
+    <row r="99" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B99" s="40"/>
+      <c r="C99" s="40"/>
+    </row>
+    <row r="100" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B100" s="40"/>
+      <c r="C100" s="40"/>
+    </row>
+  </sheetData>
+  <mergeCells count="86">
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="I14:M14"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B67:C67"/>
+    <mergeCell ref="B68:C68"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="B88:C88"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B94:C94"/>
+    <mergeCell ref="B100:C100"/>
+    <mergeCell ref="B95:C95"/>
+    <mergeCell ref="B96:C96"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B98:C98"/>
+    <mergeCell ref="B99:C99"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>